<commit_message>
Admin: publish reviewed Excel adjustments
</commit_message>
<xml_diff>
--- a/F1_Standings.xlsx
+++ b/F1_Standings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ruiro\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{106D94E8-A957-4B1B-8644-5F79E7E3A121}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29E72F94-189A-411C-9726-91763DF3CA43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Leagues" sheetId="10" r:id="rId1"/>
@@ -63491,7 +63491,7 @@
         <v>6</v>
       </c>
       <c r="E1846" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F1846" t="s">
         <v>116</v>
@@ -63526,7 +63526,7 @@
         <v>6</v>
       </c>
       <c r="E1847" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F1847" t="s">
         <v>116</v>
@@ -63558,7 +63558,7 @@
         <v>6</v>
       </c>
       <c r="E1848" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F1848" t="s">
         <v>116</v>
@@ -63590,7 +63590,7 @@
         <v>6</v>
       </c>
       <c r="E1849" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F1849" t="s">
         <v>116</v>
@@ -63622,7 +63622,7 @@
         <v>6</v>
       </c>
       <c r="E1850" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F1850" t="s">
         <v>116</v>
@@ -63654,7 +63654,7 @@
         <v>6</v>
       </c>
       <c r="E1851" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F1851" t="s">
         <v>116</v>
@@ -63686,7 +63686,7 @@
         <v>6</v>
       </c>
       <c r="E1852" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F1852" t="s">
         <v>116</v>
@@ -63718,7 +63718,7 @@
         <v>6</v>
       </c>
       <c r="E1853" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F1853" t="s">
         <v>116</v>
@@ -63750,7 +63750,7 @@
         <v>6</v>
       </c>
       <c r="E1854" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F1854" t="s">
         <v>116</v>
@@ -63782,7 +63782,7 @@
         <v>6</v>
       </c>
       <c r="E1855" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F1855" t="s">
         <v>116</v>
@@ -63814,7 +63814,7 @@
         <v>6</v>
       </c>
       <c r="E1856" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F1856" t="s">
         <v>116</v>
@@ -63846,7 +63846,7 @@
         <v>6</v>
       </c>
       <c r="E1857" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F1857" t="s">
         <v>116</v>
@@ -63878,7 +63878,7 @@
         <v>6</v>
       </c>
       <c r="E1858" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F1858" t="s">
         <v>116</v>
@@ -63910,7 +63910,7 @@
         <v>6</v>
       </c>
       <c r="E1859" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F1859" t="s">
         <v>116</v>
@@ -63942,7 +63942,7 @@
         <v>6</v>
       </c>
       <c r="E1860" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F1860" t="s">
         <v>116</v>
@@ -63974,7 +63974,7 @@
         <v>6</v>
       </c>
       <c r="E1861" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F1861" t="s">
         <v>116</v>
@@ -64006,7 +64006,7 @@
         <v>6</v>
       </c>
       <c r="E1862" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F1862" t="s">
         <v>116</v>
@@ -64038,7 +64038,7 @@
         <v>6</v>
       </c>
       <c r="E1863" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F1863" t="s">
         <v>116</v>
@@ -64073,7 +64073,7 @@
         <v>6</v>
       </c>
       <c r="E1864" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F1864" t="s">
         <v>116</v>
@@ -64105,7 +64105,7 @@
         <v>6</v>
       </c>
       <c r="E1865" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F1865" t="s">
         <v>116</v>
@@ -64137,7 +64137,7 @@
         <v>6</v>
       </c>
       <c r="E1866" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F1866" t="s">
         <v>116</v>
@@ -64172,7 +64172,7 @@
         <v>6</v>
       </c>
       <c r="E1867" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F1867" t="s">
         <v>116</v>

</xml_diff>

<commit_message>
Update Canadian Sprint and Race results from supplied workbook
</commit_message>
<xml_diff>
--- a/F1_Standings.xlsx
+++ b/F1_Standings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ruiro\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29E72F94-189A-411C-9726-91763DF3CA43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8606141A-2CDE-4C30-951C-61039481B922}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -62784,7 +62784,7 @@
         <v>204</v>
       </c>
       <c r="D1824">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1824" t="s">
         <v>207</v>
@@ -62816,7 +62816,7 @@
         <v>204</v>
       </c>
       <c r="D1825">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1825" t="s">
         <v>207</v>
@@ -62848,7 +62848,7 @@
         <v>204</v>
       </c>
       <c r="D1826">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1826" t="s">
         <v>207</v>
@@ -62880,7 +62880,7 @@
         <v>204</v>
       </c>
       <c r="D1827">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1827" t="s">
         <v>207</v>
@@ -62912,7 +62912,7 @@
         <v>204</v>
       </c>
       <c r="D1828">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1828" t="s">
         <v>207</v>
@@ -62944,7 +62944,7 @@
         <v>204</v>
       </c>
       <c r="D1829">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1829" t="s">
         <v>207</v>
@@ -62976,7 +62976,7 @@
         <v>204</v>
       </c>
       <c r="D1830">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1830" t="s">
         <v>207</v>
@@ -63008,7 +63008,7 @@
         <v>204</v>
       </c>
       <c r="D1831">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1831" t="s">
         <v>207</v>
@@ -63040,7 +63040,7 @@
         <v>204</v>
       </c>
       <c r="D1832">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1832" t="s">
         <v>207</v>
@@ -63072,7 +63072,7 @@
         <v>204</v>
       </c>
       <c r="D1833">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1833" t="s">
         <v>207</v>
@@ -63104,7 +63104,7 @@
         <v>204</v>
       </c>
       <c r="D1834">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1834" t="s">
         <v>207</v>
@@ -63136,7 +63136,7 @@
         <v>204</v>
       </c>
       <c r="D1835">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1835" t="s">
         <v>207</v>
@@ -63168,7 +63168,7 @@
         <v>204</v>
       </c>
       <c r="D1836">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1836" t="s">
         <v>207</v>
@@ -63200,7 +63200,7 @@
         <v>204</v>
       </c>
       <c r="D1837">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1837" t="s">
         <v>207</v>
@@ -63232,7 +63232,7 @@
         <v>204</v>
       </c>
       <c r="D1838">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1838" t="s">
         <v>207</v>
@@ -63264,7 +63264,7 @@
         <v>204</v>
       </c>
       <c r="D1839">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1839" t="s">
         <v>207</v>
@@ -63296,7 +63296,7 @@
         <v>204</v>
       </c>
       <c r="D1840">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1840" t="s">
         <v>207</v>
@@ -63328,7 +63328,7 @@
         <v>204</v>
       </c>
       <c r="D1841">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1841" t="s">
         <v>207</v>
@@ -63360,7 +63360,7 @@
         <v>204</v>
       </c>
       <c r="D1842">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1842" t="s">
         <v>207</v>
@@ -63392,7 +63392,7 @@
         <v>204</v>
       </c>
       <c r="D1843">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1843" t="s">
         <v>207</v>
@@ -63424,7 +63424,7 @@
         <v>204</v>
       </c>
       <c r="D1844">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1844" t="s">
         <v>207</v>
@@ -63456,7 +63456,7 @@
         <v>204</v>
       </c>
       <c r="D1845">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1845" t="s">
         <v>207</v>
@@ -63488,7 +63488,7 @@
         <v>204</v>
       </c>
       <c r="D1846">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1846" t="s">
         <v>206</v>
@@ -63523,7 +63523,7 @@
         <v>204</v>
       </c>
       <c r="D1847">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1847" t="s">
         <v>206</v>
@@ -63555,7 +63555,7 @@
         <v>204</v>
       </c>
       <c r="D1848">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1848" t="s">
         <v>206</v>
@@ -63587,7 +63587,7 @@
         <v>204</v>
       </c>
       <c r="D1849">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1849" t="s">
         <v>206</v>
@@ -63619,7 +63619,7 @@
         <v>204</v>
       </c>
       <c r="D1850">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1850" t="s">
         <v>206</v>
@@ -63651,7 +63651,7 @@
         <v>204</v>
       </c>
       <c r="D1851">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1851" t="s">
         <v>206</v>
@@ -63683,7 +63683,7 @@
         <v>204</v>
       </c>
       <c r="D1852">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1852" t="s">
         <v>206</v>
@@ -63715,7 +63715,7 @@
         <v>204</v>
       </c>
       <c r="D1853">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1853" t="s">
         <v>206</v>
@@ -63747,7 +63747,7 @@
         <v>204</v>
       </c>
       <c r="D1854">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1854" t="s">
         <v>206</v>
@@ -63779,7 +63779,7 @@
         <v>204</v>
       </c>
       <c r="D1855">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1855" t="s">
         <v>206</v>
@@ -63811,7 +63811,7 @@
         <v>204</v>
       </c>
       <c r="D1856">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1856" t="s">
         <v>206</v>
@@ -63843,7 +63843,7 @@
         <v>204</v>
       </c>
       <c r="D1857">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1857" t="s">
         <v>206</v>
@@ -63875,7 +63875,7 @@
         <v>204</v>
       </c>
       <c r="D1858">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1858" t="s">
         <v>206</v>
@@ -63907,7 +63907,7 @@
         <v>204</v>
       </c>
       <c r="D1859">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1859" t="s">
         <v>206</v>
@@ -63939,7 +63939,7 @@
         <v>204</v>
       </c>
       <c r="D1860">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1860" t="s">
         <v>206</v>
@@ -63971,7 +63971,7 @@
         <v>204</v>
       </c>
       <c r="D1861">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1861" t="s">
         <v>206</v>
@@ -64003,7 +64003,7 @@
         <v>204</v>
       </c>
       <c r="D1862">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1862" t="s">
         <v>206</v>
@@ -64035,7 +64035,7 @@
         <v>204</v>
       </c>
       <c r="D1863">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1863" t="s">
         <v>206</v>
@@ -64070,7 +64070,7 @@
         <v>204</v>
       </c>
       <c r="D1864">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1864" t="s">
         <v>206</v>
@@ -64102,7 +64102,7 @@
         <v>204</v>
       </c>
       <c r="D1865">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1865" t="s">
         <v>206</v>
@@ -64134,7 +64134,7 @@
         <v>204</v>
       </c>
       <c r="D1866">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1866" t="s">
         <v>206</v>
@@ -64169,7 +64169,7 @@
         <v>204</v>
       </c>
       <c r="D1867">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1867" t="s">
         <v>206</v>

</xml_diff>

<commit_message>
Reschedule Teikirise Azerbaijan GP to 10 January 2027
</commit_message>
<xml_diff>
--- a/F1_Standings.xlsx
+++ b/F1_Standings.xlsx
@@ -88268,14 +88268,14 @@
         <v>8</v>
       </c>
       <c r="C28" s="8">
-        <v>46292</v>
-      </c>
-      <c r="D28" s="6" t="s">
-        <v>119</v>
+        <v>46299</v>
+      </c>
+      <c r="D28" t="s">
+        <v>17</v>
       </c>
       <c r="E28" t="str">
         <f t="shared" si="5"/>
-        <v>Baku City Circuit</v>
+        <v>Suzuka International Racing Course</v>
       </c>
       <c r="F28" t="s">
         <v>191</v>
@@ -88299,14 +88299,14 @@
         <v>9</v>
       </c>
       <c r="C29" s="8">
-        <v>46299</v>
-      </c>
-      <c r="D29" t="s">
-        <v>17</v>
+        <v>46306</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>166</v>
       </c>
       <c r="E29" t="str">
         <f t="shared" si="5"/>
-        <v>Suzuka International Racing Course</v>
+        <v>Marina Bay Street Circuit</v>
       </c>
       <c r="F29" t="s">
         <v>191</v>
@@ -88330,14 +88330,14 @@
         <v>10</v>
       </c>
       <c r="C30" s="8">
-        <v>46306</v>
-      </c>
-      <c r="D30" s="6" t="s">
-        <v>166</v>
+        <v>46313</v>
+      </c>
+      <c r="D30" t="s">
+        <v>120</v>
       </c>
       <c r="E30" t="str">
         <f t="shared" si="5"/>
-        <v>Marina Bay Street Circuit</v>
+        <v>Algarve International Circuit</v>
       </c>
       <c r="F30" t="s">
         <v>191</v>
@@ -88361,14 +88361,14 @@
         <v>11</v>
       </c>
       <c r="C31" s="8">
-        <v>46313</v>
-      </c>
-      <c r="D31" t="s">
-        <v>120</v>
+        <v>46320</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>117</v>
       </c>
       <c r="E31" t="str">
         <f t="shared" ref="E31" si="6">VLOOKUP(D31,$K$1:$L$43,2,FALSE)</f>
-        <v>Algarve International Circuit</v>
+        <v>Circuit of the Americas</v>
       </c>
       <c r="F31" t="s">
         <v>191</v>
@@ -88392,14 +88392,14 @@
         <v>12</v>
       </c>
       <c r="C32" s="8">
-        <v>46320</v>
+        <v>46327</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>117</v>
+        <v>169</v>
       </c>
       <c r="E32" t="str">
         <f t="shared" si="5"/>
-        <v>Circuit of the Americas</v>
+        <v>Autódromo Hermanos Rodríguez</v>
       </c>
       <c r="F32" t="s">
         <v>191</v>
@@ -88423,14 +88423,14 @@
         <v>13</v>
       </c>
       <c r="C33" s="8">
-        <v>46327</v>
+        <v>46334</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="E33" t="str">
         <f t="shared" si="5"/>
-        <v>Autódromo Hermanos Rodríguez</v>
+        <v>Autódromo José Carlos Pace (Interlagos)</v>
       </c>
       <c r="F33" t="s">
         <v>191</v>
@@ -88454,14 +88454,14 @@
         <v>14</v>
       </c>
       <c r="C34" s="8">
-        <v>46334</v>
-      </c>
-      <c r="D34" s="6" t="s">
-        <v>171</v>
+        <v>46341</v>
+      </c>
+      <c r="D34" t="s">
+        <v>123</v>
       </c>
       <c r="E34" t="str">
         <f t="shared" si="5"/>
-        <v>Autódromo José Carlos Pace (Interlagos)</v>
+        <v>Red Bull Ring</v>
       </c>
       <c r="F34" t="s">
         <v>191</v>
@@ -88485,14 +88485,14 @@
         <v>15</v>
       </c>
       <c r="C35" s="8">
-        <v>46341</v>
-      </c>
-      <c r="D35" t="s">
-        <v>123</v>
+        <v>46348</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>115</v>
       </c>
       <c r="E35" t="str">
         <f t="shared" si="5"/>
-        <v>Red Bull Ring</v>
+        <v>Las Vegas Strip Circuit</v>
       </c>
       <c r="F35" t="s">
         <v>191</v>
@@ -88510,14 +88510,14 @@
         <v>16</v>
       </c>
       <c r="C36" s="8">
-        <v>46348</v>
+        <v>46355</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="E36" t="str">
         <f t="shared" si="5"/>
-        <v>Las Vegas Strip Circuit</v>
+        <v>Lusail International Circuit</v>
       </c>
       <c r="F36" t="s">
         <v>191</v>
@@ -88535,14 +88535,14 @@
         <v>17</v>
       </c>
       <c r="C37" s="8">
-        <v>46355</v>
+        <v>46362</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="E37" t="str">
         <f t="shared" si="5"/>
-        <v>Lusail International Circuit</v>
+        <v>Yas Marina Circuit</v>
       </c>
       <c r="F37" t="s">
         <v>191</v>
@@ -88560,14 +88560,14 @@
         <v>18</v>
       </c>
       <c r="C38" s="8">
-        <v>46362</v>
-      </c>
-      <c r="D38" s="6" t="s">
-        <v>126</v>
+        <v>46369</v>
+      </c>
+      <c r="D38" t="s">
+        <v>125</v>
       </c>
       <c r="E38" t="str">
         <f t="shared" si="5"/>
-        <v>Yas Marina Circuit</v>
+        <v>Circuit Zandvoort</v>
       </c>
       <c r="F38" t="s">
         <v>191</v>
@@ -88585,14 +88585,14 @@
         <v>19</v>
       </c>
       <c r="C39" s="8">
-        <v>46369</v>
+        <v>46376</v>
       </c>
       <c r="D39" t="s">
-        <v>125</v>
+        <v>163</v>
       </c>
       <c r="E39" t="str">
         <f t="shared" si="5"/>
-        <v>Circuit Zandvoort</v>
+        <v>Autodromo Nazionale Monza</v>
       </c>
       <c r="F39" t="s">
         <v>191</v>
@@ -88610,14 +88610,14 @@
         <v>20</v>
       </c>
       <c r="C40" s="8">
-        <v>46376</v>
+        <v>46383</v>
       </c>
       <c r="D40" t="s">
-        <v>163</v>
+        <v>113</v>
       </c>
       <c r="E40" t="str">
         <f t="shared" si="5"/>
-        <v>Autodromo Nazionale Monza</v>
+        <v>Madring</v>
       </c>
       <c r="F40" t="s">
         <v>191</v>
@@ -88635,14 +88635,14 @@
         <v>21</v>
       </c>
       <c r="C41" s="8">
-        <v>46383</v>
+        <v>46390</v>
       </c>
       <c r="D41" t="s">
-        <v>113</v>
+        <v>20</v>
       </c>
       <c r="E41" t="str">
         <f t="shared" si="5"/>
-        <v>Madring</v>
+        <v>Miami International Autodrome</v>
       </c>
       <c r="F41" t="s">
         <v>191</v>
@@ -88660,14 +88660,14 @@
         <v>22</v>
       </c>
       <c r="C42" s="8">
-        <v>46390</v>
-      </c>
-      <c r="D42" t="s">
-        <v>20</v>
+        <v>46397</v>
+      </c>
+      <c r="D42" s="6" t="s">
+        <v>119</v>
       </c>
       <c r="E42" t="str">
         <f t="shared" ref="E42" si="7">VLOOKUP(D42,$K$1:$L$43,2,FALSE)</f>
-        <v>Miami International Autodrome</v>
+        <v>Baku City Circuit</v>
       </c>
       <c r="F42" t="s">
         <v>191</v>

</xml_diff>

<commit_message>
Add Teikirise Emilia Romagna and Bahrain GPs in January 2027
</commit_message>
<xml_diff>
--- a/F1_Standings.xlsx
+++ b/F1_Standings.xlsx
@@ -88677,12 +88677,54 @@
       </c>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="C43" s="8"/>
-      <c r="G43" s="11"/>
+      <c r="A43" t="str">
+        <v>Teikirise</v>
+      </c>
+      <c r="B43" t="n">
+        <f>B42+1</f>
+        <v>23</v>
+      </c>
+      <c r="C43" t="n" s="8">
+        <v>46404</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Emilia Romagna GP</v>
+      </c>
+      <c r="E43" t="str">
+        <f>VLOOKUP(D43,$K$1:$L$43,2,FALSE)</f>
+        <v>Autodromo Enzo e Dino Ferrari (Imola)</v>
+      </c>
+      <c r="F43" t="str">
+        <v>Upcoming</v>
+      </c>
+      <c r="G43" t="n" s="11">
+        <v>0.25</v>
+      </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="C44" s="8"/>
-      <c r="G44" s="11"/>
+      <c r="A44" t="str">
+        <v>Teikirise</v>
+      </c>
+      <c r="B44" t="n">
+        <f>B43+1</f>
+        <v>24</v>
+      </c>
+      <c r="C44" t="n" s="8">
+        <v>46411</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Bahrain GP</v>
+      </c>
+      <c r="E44" t="str">
+        <f>VLOOKUP(D44,$K$1:$L$43,2,FALSE)</f>
+        <v>Bahrain International Circuit</v>
+      </c>
+      <c r="F44" t="str">
+        <v>Upcoming</v>
+      </c>
+      <c r="G44" t="n" s="11">
+        <v>0.25</v>
+      </c>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.45">
       <c r="C45" s="8"/>

</xml_diff>

<commit_message>
Import R results: Japanese GP (round 8)
</commit_message>
<xml_diff>
--- a/F1_Standings.xlsx
+++ b/F1_Standings.xlsx
@@ -64194,179 +64194,1235 @@
       </c>
     </row>
     <row r="1868" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="F1868" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1868" t="s">
-        <v>37</v>
+      <c r="A1868" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1868" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1868" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1868">
+        <v>8</v>
+      </c>
+      <c r="E1868" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1868" t="inlineStr">
+        <is>
+          <t>Japanese GP</t>
+        </is>
+      </c>
+      <c r="G1868" t="inlineStr">
+        <is>
+          <t>TomasRodri21</t>
+        </is>
+      </c>
+      <c r="H1868" t="inlineStr">
+        <is>
+          <t>McLaren</t>
+        </is>
+      </c>
+      <c r="I1868">
+        <v>1</v>
+      </c>
+      <c r="J1868">
+        <v>25</v>
+      </c>
+      <c r="K1868" t="inlineStr">
+        <is>
+          <t>88:56.869</t>
+        </is>
+      </c>
+      <c r="L1868" t="inlineStr">
+        <is>
+          <t>1:33.169</t>
+        </is>
       </c>
     </row>
     <row r="1869" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="F1869" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1869" t="s">
-        <v>37</v>
+      <c r="A1869" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1869" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1869" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1869">
+        <v>8</v>
+      </c>
+      <c r="E1869" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1869" t="inlineStr">
+        <is>
+          <t>Japanese GP</t>
+        </is>
+      </c>
+      <c r="G1869" t="inlineStr">
+        <is>
+          <t>Fatacuida</t>
+        </is>
+      </c>
+      <c r="H1869" t="inlineStr">
+        <is>
+          <t>Mercedes</t>
+        </is>
+      </c>
+      <c r="I1869">
+        <v>2</v>
+      </c>
+      <c r="J1869">
+        <v>18</v>
+      </c>
+      <c r="K1869" t="inlineStr">
+        <is>
+          <t>+11.242</t>
+        </is>
+      </c>
+      <c r="L1869" t="inlineStr">
+        <is>
+          <t>1:34.042</t>
+        </is>
       </c>
     </row>
     <row r="1870" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="F1870" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1870" t="s">
-        <v>37</v>
+      <c r="A1870" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1870" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1870" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1870">
+        <v>8</v>
+      </c>
+      <c r="E1870" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1870" t="inlineStr">
+        <is>
+          <t>Japanese GP</t>
+        </is>
+      </c>
+      <c r="G1870" t="inlineStr">
+        <is>
+          <t>Max Verstappen</t>
+        </is>
+      </c>
+      <c r="H1870" t="inlineStr">
+        <is>
+          <t>Red Bull</t>
+        </is>
+      </c>
+      <c r="I1870">
+        <v>3</v>
+      </c>
+      <c r="J1870">
+        <v>15</v>
+      </c>
+      <c r="K1870" t="inlineStr">
+        <is>
+          <t>+18.485</t>
+        </is>
+      </c>
+      <c r="L1870" t="inlineStr">
+        <is>
+          <t>1:35.476</t>
+        </is>
       </c>
     </row>
     <row r="1871" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="F1871" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1871" t="s">
-        <v>37</v>
+      <c r="A1871" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1871" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1871" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1871">
+        <v>8</v>
+      </c>
+      <c r="E1871" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1871" t="inlineStr">
+        <is>
+          <t>Japanese GP</t>
+        </is>
+      </c>
+      <c r="G1871" t="inlineStr">
+        <is>
+          <t>Charles Leclerc</t>
+        </is>
+      </c>
+      <c r="H1871" t="inlineStr">
+        <is>
+          <t>Ferrari</t>
+        </is>
+      </c>
+      <c r="I1871">
+        <v>4</v>
+      </c>
+      <c r="J1871">
+        <v>12</v>
+      </c>
+      <c r="K1871" t="inlineStr">
+        <is>
+          <t>+24.428</t>
+        </is>
+      </c>
+      <c r="L1871" t="inlineStr">
+        <is>
+          <t>1:35.329</t>
+        </is>
       </c>
     </row>
     <row r="1872" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="F1872" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1872" t="s">
-        <v>37</v>
+      <c r="A1872" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1872" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1872" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1872">
+        <v>8</v>
+      </c>
+      <c r="E1872" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1872" t="inlineStr">
+        <is>
+          <t>Japanese GP</t>
+        </is>
+      </c>
+      <c r="G1872" t="inlineStr">
+        <is>
+          <t>Carlos Sainz Jr.</t>
+        </is>
+      </c>
+      <c r="H1872" t="inlineStr">
+        <is>
+          <t>Williams</t>
+        </is>
+      </c>
+      <c r="I1872">
+        <v>5</v>
+      </c>
+      <c r="J1872">
+        <v>10</v>
+      </c>
+      <c r="K1872" t="inlineStr">
+        <is>
+          <t>+29.581</t>
+        </is>
+      </c>
+      <c r="L1872" t="inlineStr">
+        <is>
+          <t>1:35.906</t>
+        </is>
       </c>
     </row>
     <row r="1873" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1873" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1873" t="s">
-        <v>37</v>
+      <c r="A1873" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1873" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1873" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1873">
+        <v>8</v>
+      </c>
+      <c r="E1873" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1873" t="inlineStr">
+        <is>
+          <t>Japanese GP</t>
+        </is>
+      </c>
+      <c r="G1873" t="inlineStr">
+        <is>
+          <t>Alexander Albon</t>
+        </is>
+      </c>
+      <c r="H1873" t="inlineStr">
+        <is>
+          <t>Williams</t>
+        </is>
+      </c>
+      <c r="I1873">
+        <v>6</v>
+      </c>
+      <c r="J1873">
+        <v>8</v>
+      </c>
+      <c r="K1873" t="inlineStr">
+        <is>
+          <t>+31.063</t>
+        </is>
+      </c>
+      <c r="L1873" t="inlineStr">
+        <is>
+          <t>1:36.226</t>
+        </is>
       </c>
     </row>
     <row r="1874" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1874" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1874" t="s">
-        <v>37</v>
+      <c r="A1874" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1874" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1874" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1874">
+        <v>8</v>
+      </c>
+      <c r="E1874" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1874" t="inlineStr">
+        <is>
+          <t>Japanese GP</t>
+        </is>
+      </c>
+      <c r="G1874" t="inlineStr">
+        <is>
+          <t>Lewis Hamilton</t>
+        </is>
+      </c>
+      <c r="H1874" t="inlineStr">
+        <is>
+          <t>Ferrari</t>
+        </is>
+      </c>
+      <c r="I1874">
+        <v>7</v>
+      </c>
+      <c r="J1874">
+        <v>6</v>
+      </c>
+      <c r="K1874" t="inlineStr">
+        <is>
+          <t>+39.035</t>
+        </is>
+      </c>
+      <c r="L1874" t="inlineStr">
+        <is>
+          <t>1:37.026</t>
+        </is>
       </c>
     </row>
     <row r="1875" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1875" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1875" t="s">
-        <v>37</v>
+      <c r="A1875" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1875" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1875" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1875">
+        <v>8</v>
+      </c>
+      <c r="E1875" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1875" t="inlineStr">
+        <is>
+          <t>Japanese GP</t>
+        </is>
+      </c>
+      <c r="G1875" t="inlineStr">
+        <is>
+          <t>Fernando Alonso</t>
+        </is>
+      </c>
+      <c r="H1875" t="inlineStr">
+        <is>
+          <t>Aston Martin</t>
+        </is>
+      </c>
+      <c r="I1875">
+        <v>8</v>
+      </c>
+      <c r="J1875">
+        <v>4</v>
+      </c>
+      <c r="K1875" t="inlineStr">
+        <is>
+          <t>+39.430</t>
+        </is>
+      </c>
+      <c r="L1875" t="inlineStr">
+        <is>
+          <t>1:36.685</t>
+        </is>
       </c>
     </row>
     <row r="1876" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1876" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1876" t="s">
-        <v>37</v>
+      <c r="A1876" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1876" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1876" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1876">
+        <v>8</v>
+      </c>
+      <c r="E1876" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1876" t="inlineStr">
+        <is>
+          <t>Japanese GP</t>
+        </is>
+      </c>
+      <c r="G1876" t="inlineStr">
+        <is>
+          <t>Franco Colapinto</t>
+        </is>
+      </c>
+      <c r="H1876" t="inlineStr">
+        <is>
+          <t>Alpine</t>
+        </is>
+      </c>
+      <c r="I1876">
+        <v>9</v>
+      </c>
+      <c r="J1876">
+        <v>2</v>
+      </c>
+      <c r="K1876" t="inlineStr">
+        <is>
+          <t>+44.676</t>
+        </is>
+      </c>
+      <c r="L1876" t="inlineStr">
+        <is>
+          <t>1:37.128</t>
+        </is>
       </c>
     </row>
     <row r="1877" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1877" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1877" t="s">
-        <v>37</v>
+      <c r="A1877" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1877" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1877" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1877">
+        <v>8</v>
+      </c>
+      <c r="E1877" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1877" t="inlineStr">
+        <is>
+          <t>Japanese GP</t>
+        </is>
+      </c>
+      <c r="G1877" t="inlineStr">
+        <is>
+          <t>Kimi Antonelli</t>
+        </is>
+      </c>
+      <c r="H1877" t="inlineStr">
+        <is>
+          <t>Mercedes</t>
+        </is>
+      </c>
+      <c r="I1877">
+        <v>10</v>
+      </c>
+      <c r="J1877">
+        <v>1</v>
+      </c>
+      <c r="K1877" t="inlineStr">
+        <is>
+          <t>+44.869</t>
+        </is>
+      </c>
+      <c r="L1877" t="inlineStr">
+        <is>
+          <t>1:37.212</t>
+        </is>
       </c>
     </row>
     <row r="1878" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1878" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1878" t="s">
-        <v>37</v>
+      <c r="A1878" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1878" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1878" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1878">
+        <v>8</v>
+      </c>
+      <c r="E1878" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1878" t="inlineStr">
+        <is>
+          <t>Japanese GP</t>
+        </is>
+      </c>
+      <c r="G1878" t="inlineStr">
+        <is>
+          <t>Arvid Lidblad</t>
+        </is>
+      </c>
+      <c r="H1878" t="inlineStr">
+        <is>
+          <t>Racing Bulls</t>
+        </is>
+      </c>
+      <c r="I1878">
+        <v>11</v>
+      </c>
+      <c r="J1878">
+        <v>0</v>
+      </c>
+      <c r="K1878" t="inlineStr">
+        <is>
+          <t>+44.934</t>
+        </is>
+      </c>
+      <c r="L1878" t="inlineStr">
+        <is>
+          <t>1:37.293</t>
+        </is>
       </c>
     </row>
     <row r="1879" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1879" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1879" t="s">
-        <v>37</v>
+      <c r="A1879" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1879" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1879" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1879">
+        <v>8</v>
+      </c>
+      <c r="E1879" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1879" t="inlineStr">
+        <is>
+          <t>Japanese GP</t>
+        </is>
+      </c>
+      <c r="G1879" t="inlineStr">
+        <is>
+          <t>Liam Lawson</t>
+        </is>
+      </c>
+      <c r="H1879" t="inlineStr">
+        <is>
+          <t>Racing Bulls</t>
+        </is>
+      </c>
+      <c r="I1879">
+        <v>12</v>
+      </c>
+      <c r="J1879">
+        <v>0</v>
+      </c>
+      <c r="K1879" t="inlineStr">
+        <is>
+          <t>+46.047</t>
+        </is>
+      </c>
+      <c r="L1879" t="inlineStr">
+        <is>
+          <t>1:37.178</t>
+        </is>
       </c>
     </row>
     <row r="1880" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1880" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1880" t="s">
-        <v>37</v>
+      <c r="A1880" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1880" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1880" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1880">
+        <v>8</v>
+      </c>
+      <c r="E1880" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1880" t="inlineStr">
+        <is>
+          <t>Japanese GP</t>
+        </is>
+      </c>
+      <c r="G1880" t="inlineStr">
+        <is>
+          <t>Oliver Bearman</t>
+        </is>
+      </c>
+      <c r="H1880" t="inlineStr">
+        <is>
+          <t>Haas</t>
+        </is>
+      </c>
+      <c r="I1880">
+        <v>13</v>
+      </c>
+      <c r="J1880">
+        <v>0</v>
+      </c>
+      <c r="K1880" t="inlineStr">
+        <is>
+          <t>+1 Lap</t>
+        </is>
+      </c>
+      <c r="L1880" t="inlineStr">
+        <is>
+          <t>1:36.028</t>
+        </is>
       </c>
     </row>
     <row r="1881" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1881" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1881" t="s">
-        <v>37</v>
+      <c r="A1881" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1881" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1881" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1881">
+        <v>8</v>
+      </c>
+      <c r="E1881" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1881" t="inlineStr">
+        <is>
+          <t>Japanese GP</t>
+        </is>
+      </c>
+      <c r="G1881" t="inlineStr">
+        <is>
+          <t>Esteban Ocon</t>
+        </is>
+      </c>
+      <c r="H1881" t="inlineStr">
+        <is>
+          <t>Haas</t>
+        </is>
+      </c>
+      <c r="I1881">
+        <v>14</v>
+      </c>
+      <c r="J1881">
+        <v>0</v>
+      </c>
+      <c r="K1881" t="inlineStr">
+        <is>
+          <t>+1 Lap</t>
+        </is>
+      </c>
+      <c r="L1881" t="inlineStr">
+        <is>
+          <t>1:35.840</t>
+        </is>
       </c>
     </row>
     <row r="1882" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1882" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1882" t="s">
-        <v>37</v>
+      <c r="A1882" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1882" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1882" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1882">
+        <v>8</v>
+      </c>
+      <c r="E1882" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1882" t="inlineStr">
+        <is>
+          <t>Japanese GP</t>
+        </is>
+      </c>
+      <c r="G1882" t="inlineStr">
+        <is>
+          <t>Nico Hülkenberg</t>
+        </is>
+      </c>
+      <c r="H1882" t="inlineStr">
+        <is>
+          <t>Audi</t>
+        </is>
+      </c>
+      <c r="I1882">
+        <v>15</v>
+      </c>
+      <c r="J1882">
+        <v>0</v>
+      </c>
+      <c r="K1882" t="inlineStr">
+        <is>
+          <t>+1 Lap</t>
+        </is>
+      </c>
+      <c r="L1882" t="inlineStr">
+        <is>
+          <t>1:37.347</t>
+        </is>
       </c>
     </row>
     <row r="1883" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1883" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1883" t="s">
-        <v>37</v>
+      <c r="A1883" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1883" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1883" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1883">
+        <v>8</v>
+      </c>
+      <c r="E1883" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1883" t="inlineStr">
+        <is>
+          <t>Japanese GP</t>
+        </is>
+      </c>
+      <c r="G1883" t="inlineStr">
+        <is>
+          <t>Valtteri Bottas</t>
+        </is>
+      </c>
+      <c r="H1883" t="inlineStr">
+        <is>
+          <t>Cadillac</t>
+        </is>
+      </c>
+      <c r="I1883">
+        <v>16</v>
+      </c>
+      <c r="J1883">
+        <v>0</v>
+      </c>
+      <c r="K1883" t="inlineStr">
+        <is>
+          <t>+1 Lap</t>
+        </is>
+      </c>
+      <c r="L1883" t="inlineStr">
+        <is>
+          <t>1:37.179</t>
+        </is>
       </c>
     </row>
     <row r="1884" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1884" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1884" t="s">
-        <v>37</v>
+      <c r="A1884" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1884" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1884" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1884">
+        <v>8</v>
+      </c>
+      <c r="E1884" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1884" t="inlineStr">
+        <is>
+          <t>Japanese GP</t>
+        </is>
+      </c>
+      <c r="G1884" t="inlineStr">
+        <is>
+          <t>Lance Stroll</t>
+        </is>
+      </c>
+      <c r="H1884" t="inlineStr">
+        <is>
+          <t>Aston Martin</t>
+        </is>
+      </c>
+      <c r="I1884">
+        <v>17</v>
+      </c>
+      <c r="J1884">
+        <v>0</v>
+      </c>
+      <c r="K1884" t="inlineStr">
+        <is>
+          <t>+1 Lap</t>
+        </is>
+      </c>
+      <c r="L1884" t="inlineStr">
+        <is>
+          <t>1:37.916</t>
+        </is>
       </c>
     </row>
     <row r="1885" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1885" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1885" t="s">
-        <v>37</v>
+      <c r="A1885" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1885" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1885" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1885">
+        <v>8</v>
+      </c>
+      <c r="E1885" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1885" t="inlineStr">
+        <is>
+          <t>Japanese GP</t>
+        </is>
+      </c>
+      <c r="G1885" t="inlineStr">
+        <is>
+          <t>Gabriel Bortoleto</t>
+        </is>
+      </c>
+      <c r="H1885" t="inlineStr">
+        <is>
+          <t>Audi</t>
+        </is>
+      </c>
+      <c r="I1885">
+        <v>18</v>
+      </c>
+      <c r="J1885">
+        <v>0</v>
+      </c>
+      <c r="K1885" t="inlineStr">
+        <is>
+          <t>+1 Lap</t>
+        </is>
+      </c>
+      <c r="L1885" t="inlineStr">
+        <is>
+          <t>1:37.930</t>
+        </is>
       </c>
     </row>
     <row r="1886" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1886" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1886" t="s">
-        <v>37</v>
+      <c r="A1886" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1886" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1886" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1886">
+        <v>8</v>
+      </c>
+      <c r="E1886" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1886" t="inlineStr">
+        <is>
+          <t>Japanese GP</t>
+        </is>
+      </c>
+      <c r="G1886" t="inlineStr">
+        <is>
+          <t>Sergio Perez</t>
+        </is>
+      </c>
+      <c r="H1886" t="inlineStr">
+        <is>
+          <t>Cadillac</t>
+        </is>
+      </c>
+      <c r="I1886">
+        <v>19</v>
+      </c>
+      <c r="J1886">
+        <v>0</v>
+      </c>
+      <c r="K1886" t="inlineStr">
+        <is>
+          <t>+1 Lap</t>
+        </is>
+      </c>
+      <c r="L1886" t="inlineStr">
+        <is>
+          <t>1:39.014</t>
+        </is>
       </c>
     </row>
     <row r="1887" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1887" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1887" t="s">
-        <v>37</v>
+      <c r="A1887" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1887" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1887" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1887">
+        <v>8</v>
+      </c>
+      <c r="E1887" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1887" t="inlineStr">
+        <is>
+          <t>Japanese GP</t>
+        </is>
+      </c>
+      <c r="G1887" t="inlineStr">
+        <is>
+          <t>Polingua</t>
+        </is>
+      </c>
+      <c r="H1887" t="inlineStr">
+        <is>
+          <t>Red Bull</t>
+        </is>
+      </c>
+      <c r="I1887">
+        <v>20</v>
+      </c>
+      <c r="J1887">
+        <v>0</v>
+      </c>
+      <c r="K1887" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="L1887" t="inlineStr">
+        <is>
+          <t>1:36.147</t>
+        </is>
       </c>
     </row>
     <row r="1888" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1888" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1888" t="s">
-        <v>37</v>
+      <c r="A1888" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1888" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1888" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1888">
+        <v>8</v>
+      </c>
+      <c r="E1888" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1888" t="inlineStr">
+        <is>
+          <t>Japanese GP</t>
+        </is>
+      </c>
+      <c r="G1888" t="inlineStr">
+        <is>
+          <t>Lando Norris</t>
+        </is>
+      </c>
+      <c r="H1888" t="inlineStr">
+        <is>
+          <t>McLaren</t>
+        </is>
+      </c>
+      <c r="I1888">
+        <v>21</v>
+      </c>
+      <c r="J1888">
+        <v>0</v>
+      </c>
+      <c r="K1888" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="L1888" t="inlineStr">
+        <is>
+          <t>1:35.788</t>
+        </is>
       </c>
     </row>
     <row r="1889" spans="6:10" x14ac:dyDescent="0.45">
-      <c r="F1889" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1889" t="s">
-        <v>37</v>
+      <c r="A1889" t="inlineStr">
+        <is>
+          <t>F1 25: 2026 Season pack</t>
+        </is>
+      </c>
+      <c r="B1889" t="inlineStr">
+        <is>
+          <t>2026-T02</t>
+        </is>
+      </c>
+      <c r="C1889" t="inlineStr">
+        <is>
+          <t>Teikirise</t>
+        </is>
+      </c>
+      <c r="D1889">
+        <v>8</v>
+      </c>
+      <c r="E1889" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F1889" t="inlineStr">
+        <is>
+          <t>Japanese GP</t>
+        </is>
+      </c>
+      <c r="G1889" t="inlineStr">
+        <is>
+          <t>Pierre Gasly</t>
+        </is>
+      </c>
+      <c r="H1889" t="inlineStr">
+        <is>
+          <t>Alpine</t>
+        </is>
+      </c>
+      <c r="I1889">
+        <v>22</v>
+      </c>
+      <c r="J1889">
+        <v>0</v>
+      </c>
+      <c r="K1889" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="L1889" t="inlineStr">
+        <is>
+          <t>1:37.326</t>
+        </is>
       </c>
     </row>
     <row r="1890" spans="6:10" x14ac:dyDescent="0.45">
@@ -88277,8 +89333,10 @@
         <f t="shared" si="5"/>
         <v>Suzuka International Racing Course</v>
       </c>
-      <c r="F28" t="s">
-        <v>191</v>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
       </c>
       <c r="G28" s="11">
         <v>0.25</v>

</xml_diff>

<commit_message>
Correct round nine results to United States GP
</commit_message>
<xml_diff>
--- a/F1_Standings.xlsx
+++ b/F1_Standings.xlsx
@@ -65234,8 +65234,10 @@
       <c r="E1890" t="s">
         <v>206</v>
       </c>
-      <c r="F1890" t="s">
-        <v>17</v>
+      <c r="F1890" t="inlineStr">
+        <is>
+          <t>United States GP</t>
+        </is>
       </c>
       <c r="G1890" t="s">
         <v>32</v>
@@ -65273,8 +65275,10 @@
       <c r="E1891" t="s">
         <v>206</v>
       </c>
-      <c r="F1891" t="s">
-        <v>17</v>
+      <c r="F1891" t="inlineStr">
+        <is>
+          <t>United States GP</t>
+        </is>
       </c>
       <c r="G1891" t="s">
         <v>34</v>
@@ -65312,8 +65316,10 @@
       <c r="E1892" t="s">
         <v>206</v>
       </c>
-      <c r="F1892" t="s">
-        <v>17</v>
+      <c r="F1892" t="inlineStr">
+        <is>
+          <t>United States GP</t>
+        </is>
       </c>
       <c r="G1892" t="s">
         <v>3</v>
@@ -65351,8 +65357,10 @@
       <c r="E1893" t="s">
         <v>206</v>
       </c>
-      <c r="F1893" t="s">
-        <v>17</v>
+      <c r="F1893" t="inlineStr">
+        <is>
+          <t>United States GP</t>
+        </is>
       </c>
       <c r="G1893" t="s">
         <v>0</v>
@@ -65390,8 +65398,10 @@
       <c r="E1894" t="s">
         <v>206</v>
       </c>
-      <c r="F1894" t="s">
-        <v>17</v>
+      <c r="F1894" t="inlineStr">
+        <is>
+          <t>United States GP</t>
+        </is>
       </c>
       <c r="G1894" t="s">
         <v>1</v>
@@ -65429,8 +65439,10 @@
       <c r="E1895" t="s">
         <v>206</v>
       </c>
-      <c r="F1895" t="s">
-        <v>17</v>
+      <c r="F1895" t="inlineStr">
+        <is>
+          <t>United States GP</t>
+        </is>
       </c>
       <c r="G1895" t="s">
         <v>2</v>
@@ -65468,8 +65480,10 @@
       <c r="E1896" t="s">
         <v>206</v>
       </c>
-      <c r="F1896" t="s">
-        <v>17</v>
+      <c r="F1896" t="inlineStr">
+        <is>
+          <t>United States GP</t>
+        </is>
       </c>
       <c r="G1896" t="s">
         <v>200</v>
@@ -65507,8 +65521,10 @@
       <c r="E1897" t="s">
         <v>206</v>
       </c>
-      <c r="F1897" t="s">
-        <v>17</v>
+      <c r="F1897" t="inlineStr">
+        <is>
+          <t>United States GP</t>
+        </is>
       </c>
       <c r="G1897" t="s">
         <v>12</v>
@@ -65546,8 +65562,10 @@
       <c r="E1898" t="s">
         <v>206</v>
       </c>
-      <c r="F1898" t="s">
-        <v>17</v>
+      <c r="F1898" t="inlineStr">
+        <is>
+          <t>United States GP</t>
+        </is>
       </c>
       <c r="G1898" t="s">
         <v>8</v>
@@ -65585,8 +65603,10 @@
       <c r="E1899" t="s">
         <v>206</v>
       </c>
-      <c r="F1899" t="s">
-        <v>17</v>
+      <c r="F1899" t="inlineStr">
+        <is>
+          <t>United States GP</t>
+        </is>
       </c>
       <c r="G1899" t="s">
         <v>5</v>
@@ -65624,8 +65644,10 @@
       <c r="E1900" t="s">
         <v>206</v>
       </c>
-      <c r="F1900" t="s">
-        <v>17</v>
+      <c r="F1900" t="inlineStr">
+        <is>
+          <t>United States GP</t>
+        </is>
       </c>
       <c r="G1900" t="s">
         <v>202</v>
@@ -65663,8 +65685,10 @@
       <c r="E1901" t="s">
         <v>206</v>
       </c>
-      <c r="F1901" t="s">
-        <v>17</v>
+      <c r="F1901" t="inlineStr">
+        <is>
+          <t>United States GP</t>
+        </is>
       </c>
       <c r="G1901" t="s">
         <v>13</v>
@@ -65702,8 +65726,10 @@
       <c r="E1902" t="s">
         <v>206</v>
       </c>
-      <c r="F1902" t="s">
-        <v>17</v>
+      <c r="F1902" t="inlineStr">
+        <is>
+          <t>United States GP</t>
+        </is>
       </c>
       <c r="G1902" t="s">
         <v>6</v>
@@ -65741,8 +65767,10 @@
       <c r="E1903" t="s">
         <v>206</v>
       </c>
-      <c r="F1903" t="s">
-        <v>17</v>
+      <c r="F1903" t="inlineStr">
+        <is>
+          <t>United States GP</t>
+        </is>
       </c>
       <c r="G1903" t="s">
         <v>14</v>
@@ -65780,8 +65808,10 @@
       <c r="E1904" t="s">
         <v>206</v>
       </c>
-      <c r="F1904" t="s">
-        <v>17</v>
+      <c r="F1904" t="inlineStr">
+        <is>
+          <t>United States GP</t>
+        </is>
       </c>
       <c r="G1904" t="s">
         <v>9</v>
@@ -65819,8 +65849,10 @@
       <c r="E1905" t="s">
         <v>206</v>
       </c>
-      <c r="F1905" t="s">
-        <v>17</v>
+      <c r="F1905" t="inlineStr">
+        <is>
+          <t>United States GP</t>
+        </is>
       </c>
       <c r="G1905" t="s">
         <v>201</v>
@@ -65858,8 +65890,10 @@
       <c r="E1906" t="s">
         <v>206</v>
       </c>
-      <c r="F1906" t="s">
-        <v>17</v>
+      <c r="F1906" t="inlineStr">
+        <is>
+          <t>United States GP</t>
+        </is>
       </c>
       <c r="G1906" t="s">
         <v>55</v>
@@ -65897,8 +65931,10 @@
       <c r="E1907" t="s">
         <v>206</v>
       </c>
-      <c r="F1907" t="s">
-        <v>17</v>
+      <c r="F1907" t="inlineStr">
+        <is>
+          <t>United States GP</t>
+        </is>
       </c>
       <c r="G1907" t="s">
         <v>79</v>
@@ -65936,8 +65972,10 @@
       <c r="E1908" t="s">
         <v>206</v>
       </c>
-      <c r="F1908" t="s">
-        <v>17</v>
+      <c r="F1908" t="inlineStr">
+        <is>
+          <t>United States GP</t>
+        </is>
       </c>
       <c r="G1908" t="s">
         <v>35</v>
@@ -65975,8 +66013,10 @@
       <c r="E1909" t="s">
         <v>206</v>
       </c>
-      <c r="F1909" t="s">
-        <v>17</v>
+      <c r="F1909" t="inlineStr">
+        <is>
+          <t>United States GP</t>
+        </is>
       </c>
       <c r="G1909" t="s">
         <v>11</v>
@@ -66014,8 +66054,10 @@
       <c r="E1910" t="s">
         <v>206</v>
       </c>
-      <c r="F1910" t="s">
-        <v>17</v>
+      <c r="F1910" t="inlineStr">
+        <is>
+          <t>United States GP</t>
+        </is>
       </c>
       <c r="G1910" t="s">
         <v>33</v>
@@ -66053,8 +66095,10 @@
       <c r="E1911" t="s">
         <v>206</v>
       </c>
-      <c r="F1911" t="s">
-        <v>17</v>
+      <c r="F1911" t="inlineStr">
+        <is>
+          <t>United States GP</t>
+        </is>
       </c>
       <c r="G1911" t="s">
         <v>10</v>

</xml_diff>